<commit_message>
feat: upload de planilha direto pelo sidebar
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Claudio\Documents\verdent-projects\new-project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/60bd3766fe3b56c0/Nova pasta/Nova pasta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FEED880-5822-4A30-B3FE-E0773491E4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2C66AA5-2F67-4010-B837-35B29476A991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F2DED76B-5FEA-48D5-9DAC-66F60A430568}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -111,7 +111,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="7" formatCode="&quot;R$&quot;\ #,##0.00;\-&quot;R$&quot;\ #,##0.00"/>
-    <numFmt numFmtId="164" formatCode="mmmm\,\ yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="mmmm\,\ yyyy;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -144,7 +144,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -246,7 +246,7 @@
             <v>109</v>
           </cell>
           <cell r="BL93">
-            <v>61</v>
+            <v>54</v>
           </cell>
         </row>
         <row r="94">
@@ -290,7 +290,7 @@
             <v>108</v>
           </cell>
           <cell r="BL94">
-            <v>88</v>
+            <v>68</v>
           </cell>
         </row>
         <row r="95">
@@ -334,7 +334,7 @@
             <v>277</v>
           </cell>
           <cell r="BL95">
-            <v>177</v>
+            <v>116</v>
           </cell>
         </row>
         <row r="96">
@@ -378,7 +378,7 @@
             <v>5</v>
           </cell>
           <cell r="BL96">
-            <v>6</v>
+            <v>4</v>
           </cell>
         </row>
         <row r="97">
@@ -422,7 +422,7 @@
             <v>40</v>
           </cell>
           <cell r="BL97">
-            <v>32</v>
+            <v>28</v>
           </cell>
         </row>
         <row r="98">
@@ -466,7 +466,7 @@
             <v>78</v>
           </cell>
           <cell r="BL98">
-            <v>70</v>
+            <v>57</v>
           </cell>
         </row>
         <row r="99">
@@ -554,7 +554,7 @@
             <v>892</v>
           </cell>
           <cell r="BL100">
-            <v>726</v>
+            <v>547</v>
           </cell>
         </row>
         <row r="101">
@@ -598,7 +598,7 @@
             <v>425</v>
           </cell>
           <cell r="BL101">
-            <v>508</v>
+            <v>390</v>
           </cell>
         </row>
         <row r="102">
@@ -642,7 +642,7 @@
             <v>775</v>
           </cell>
           <cell r="BL102">
-            <v>543</v>
+            <v>420</v>
           </cell>
         </row>
         <row r="103">
@@ -903,7 +903,7 @@
             <v>0</v>
           </cell>
           <cell r="BL120">
-            <v>1041.4000000000001</v>
+            <v>1047.4000000000001</v>
           </cell>
         </row>
         <row r="121">
@@ -953,7 +953,7 @@
             <v>523.79</v>
           </cell>
           <cell r="BL121">
-            <v>397.25</v>
+            <v>173.1</v>
           </cell>
         </row>
         <row r="122">
@@ -1003,7 +1003,7 @@
             <v>599.47</v>
           </cell>
           <cell r="BL122">
-            <v>530.91</v>
+            <v>537.89</v>
           </cell>
         </row>
         <row r="123">
@@ -1103,7 +1103,7 @@
             <v>51.99</v>
           </cell>
           <cell r="BL124">
-            <v>37.4</v>
+            <v>41.3</v>
           </cell>
         </row>
         <row r="125">
@@ -1303,7 +1303,7 @@
             <v>1664.01</v>
           </cell>
           <cell r="BL128">
-            <v>4848</v>
+            <v>217</v>
           </cell>
         </row>
         <row r="129">
@@ -1353,7 +1353,7 @@
             <v>1644.31</v>
           </cell>
           <cell r="BL129">
-            <v>2100.16</v>
+            <v>2027.17</v>
           </cell>
         </row>
         <row r="130">
@@ -1503,7 +1503,7 @@
             <v>508.18</v>
           </cell>
           <cell r="BL132">
-            <v>66.400000000000006</v>
+            <v>66.7</v>
           </cell>
         </row>
         <row r="133">
@@ -1553,7 +1553,7 @@
             <v>548.19000000000005</v>
           </cell>
           <cell r="BL133">
-            <v>737.05</v>
+            <v>114.6</v>
           </cell>
         </row>
         <row r="134">
@@ -2053,7 +2053,7 @@
             <v>0</v>
           </cell>
           <cell r="BL145">
-            <v>959.3</v>
+            <v>163</v>
           </cell>
         </row>
         <row r="146">
@@ -2103,7 +2103,7 @@
             <v>423.9</v>
           </cell>
           <cell r="BL146">
-            <v>619.61</v>
+            <v>579.05999999999995</v>
           </cell>
         </row>
         <row r="147">
@@ -2153,7 +2153,7 @@
             <v>6771.6</v>
           </cell>
           <cell r="BL147">
-            <v>994.28</v>
+            <v>907.53</v>
           </cell>
         </row>
         <row r="148">
@@ -2203,7 +2203,7 @@
             <v>1756.31</v>
           </cell>
           <cell r="BL148">
-            <v>507.14</v>
+            <v>441.39</v>
           </cell>
         </row>
         <row r="149">
@@ -2253,7 +2253,7 @@
             <v>392.52</v>
           </cell>
           <cell r="BL149">
-            <v>65.3</v>
+            <v>49.3</v>
           </cell>
         </row>
         <row r="150">
@@ -2353,7 +2353,7 @@
             <v>475.55</v>
           </cell>
           <cell r="BL151">
-            <v>51.64</v>
+            <v>29.94</v>
           </cell>
         </row>
         <row r="152">
@@ -2453,7 +2453,7 @@
             <v>6968.14</v>
           </cell>
           <cell r="BL153">
-            <v>743.18</v>
+            <v>731.48</v>
           </cell>
         </row>
         <row r="154">
@@ -2503,7 +2503,7 @@
             <v>351.6</v>
           </cell>
           <cell r="BL154">
-            <v>964.24</v>
+            <v>936.84</v>
           </cell>
         </row>
         <row r="155">
@@ -2553,7 +2553,7 @@
             <v>275.2</v>
           </cell>
           <cell r="BL155">
-            <v>334.8</v>
+            <v>281.3</v>
           </cell>
         </row>
         <row r="156">
@@ -2653,7 +2653,7 @@
             <v>1453.89</v>
           </cell>
           <cell r="BL157">
-            <v>632.67999999999995</v>
+            <v>492.81</v>
           </cell>
         </row>
         <row r="158">
@@ -2703,7 +2703,7 @@
             <v>87.73</v>
           </cell>
           <cell r="BL158">
-            <v>246.3</v>
+            <v>245.3</v>
           </cell>
         </row>
         <row r="159">
@@ -3053,7 +3053,7 @@
             <v>1528.85</v>
           </cell>
           <cell r="BL167">
-            <v>1436.72</v>
+            <v>1238.8</v>
           </cell>
         </row>
         <row r="168">
@@ -3203,7 +3203,7 @@
             <v>806.7</v>
           </cell>
           <cell r="BL170">
-            <v>699.1</v>
+            <v>579.29999999999995</v>
           </cell>
         </row>
         <row r="171">
@@ -3253,7 +3253,7 @@
             <v>2564.08</v>
           </cell>
           <cell r="BL171">
-            <v>923.53</v>
+            <v>331.3</v>
           </cell>
         </row>
         <row r="172">
@@ -3303,7 +3303,7 @@
             <v>3205.26</v>
           </cell>
           <cell r="BL172">
-            <v>1279.26</v>
+            <v>850.52</v>
           </cell>
         </row>
         <row r="173">
@@ -3353,7 +3353,7 @@
             <v>5782.77</v>
           </cell>
           <cell r="BL173">
-            <v>1377.73</v>
+            <v>882.29</v>
           </cell>
         </row>
         <row r="174">
@@ -3403,7 +3403,7 @@
             <v>360.6</v>
           </cell>
           <cell r="BL174">
-            <v>159.35</v>
+            <v>117.8</v>
           </cell>
         </row>
         <row r="175">
@@ -3503,7 +3503,7 @@
             <v>276.93</v>
           </cell>
           <cell r="BL176">
-            <v>215.83</v>
+            <v>150.47999999999999</v>
           </cell>
         </row>
         <row r="177">
@@ -3603,7 +3603,7 @@
             <v>7670.07</v>
           </cell>
           <cell r="BL178">
-            <v>4924.63</v>
+            <v>2479.83</v>
           </cell>
         </row>
         <row r="179">
@@ -3653,7 +3653,7 @@
             <v>3574.39</v>
           </cell>
           <cell r="BL179">
-            <v>2211.31</v>
+            <v>664.76</v>
           </cell>
         </row>
         <row r="180">
@@ -3703,7 +3703,7 @@
             <v>799.37</v>
           </cell>
           <cell r="BL180">
-            <v>586.82000000000005</v>
+            <v>552.47</v>
           </cell>
         </row>
         <row r="181">
@@ -3803,7 +3803,7 @@
             <v>2160.71</v>
           </cell>
           <cell r="BL182">
-            <v>2155.6799999999998</v>
+            <v>1177.83</v>
           </cell>
         </row>
         <row r="183">
@@ -3853,7 +3853,7 @@
             <v>5356.76</v>
           </cell>
           <cell r="BL183">
-            <v>2663.63</v>
+            <v>2421.7399999999998</v>
           </cell>
         </row>
         <row r="184">
@@ -4453,7 +4453,7 @@
             <v>32.49</v>
           </cell>
           <cell r="BL197">
-            <v>78.959999999999994</v>
+            <v>0.01</v>
           </cell>
         </row>
         <row r="198">
@@ -4653,7 +4653,7 @@
             <v>0</v>
           </cell>
           <cell r="BL201">
-            <v>5.56</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="202">
@@ -4803,7 +4803,7 @@
             <v>64.069999999999993</v>
           </cell>
           <cell r="BL204">
-            <v>4.96</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="205">
@@ -5553,7 +5553,7 @@
             <v>203.03</v>
           </cell>
           <cell r="BL221">
-            <v>21.49</v>
+            <v>17.89</v>
           </cell>
         </row>
         <row r="222">
@@ -5653,7 +5653,7 @@
             <v>788.08</v>
           </cell>
           <cell r="BL223">
-            <v>262.37</v>
+            <v>241.87</v>
           </cell>
         </row>
         <row r="224">
@@ -5953,7 +5953,7 @@
             <v>128.09</v>
           </cell>
           <cell r="BL229">
-            <v>460.75</v>
+            <v>466.05</v>
           </cell>
         </row>
         <row r="230">
@@ -6103,7 +6103,7 @@
             <v>347.7</v>
           </cell>
           <cell r="BL232">
-            <v>236.83</v>
+            <v>193.03</v>
           </cell>
         </row>
         <row r="233">
@@ -6703,7 +6703,7 @@
             <v>449.41</v>
           </cell>
           <cell r="BL246">
-            <v>493.17</v>
+            <v>436.87</v>
           </cell>
         </row>
         <row r="247">
@@ -6753,7 +6753,7 @@
             <v>1131.74</v>
           </cell>
           <cell r="BL247">
-            <v>354.19</v>
+            <v>304.58999999999997</v>
           </cell>
         </row>
         <row r="248">
@@ -6803,7 +6803,7 @@
             <v>989.68</v>
           </cell>
           <cell r="BL248">
-            <v>597.6</v>
+            <v>563.29999999999995</v>
           </cell>
         </row>
         <row r="249">
@@ -7053,7 +7053,7 @@
             <v>1212.5</v>
           </cell>
           <cell r="BL253">
-            <v>299.39999999999998</v>
+            <v>129.5</v>
           </cell>
         </row>
         <row r="254">
@@ -7103,7 +7103,7 @@
             <v>1217.27</v>
           </cell>
           <cell r="BL254">
-            <v>213.08</v>
+            <v>199.18</v>
           </cell>
         </row>
         <row r="255">
@@ -7253,7 +7253,7 @@
             <v>332.2</v>
           </cell>
           <cell r="BL257">
-            <v>482.65</v>
+            <v>470.95</v>
           </cell>
         </row>
         <row r="258">
@@ -7303,7 +7303,7 @@
             <v>282.8</v>
           </cell>
           <cell r="BL258">
-            <v>585.54999999999995</v>
+            <v>313.75</v>
           </cell>
         </row>
         <row r="259">
@@ -8803,7 +8803,7 @@
             <v>10911.5</v>
           </cell>
           <cell r="BL292">
-            <v>21505.040000000001</v>
+            <v>7867.21</v>
           </cell>
         </row>
         <row r="293">
@@ -8953,7 +8953,7 @@
             <v>9643.9500000000007</v>
           </cell>
           <cell r="BL295">
-            <v>5286.1</v>
+            <v>4716.7</v>
           </cell>
         </row>
         <row r="296">
@@ -9003,7 +9003,7 @@
             <v>7099.57</v>
           </cell>
           <cell r="BL296">
-            <v>9589.81</v>
+            <v>5330.29</v>
           </cell>
         </row>
         <row r="297">
@@ -9053,7 +9053,7 @@
             <v>10437.030000000001</v>
           </cell>
           <cell r="BL297">
-            <v>9748.14</v>
+            <v>8063.34</v>
           </cell>
         </row>
         <row r="298">
@@ -9103,7 +9103,7 @@
             <v>14032.28</v>
           </cell>
           <cell r="BL298">
-            <v>15233.71</v>
+            <v>10665.79</v>
           </cell>
         </row>
         <row r="299">
@@ -9153,7 +9153,7 @@
             <v>819.93</v>
           </cell>
           <cell r="BL299">
-            <v>1123.31</v>
+            <v>649.42999999999995</v>
           </cell>
         </row>
         <row r="300">
@@ -9253,7 +9253,7 @@
             <v>1498.34</v>
           </cell>
           <cell r="BL301">
-            <v>2654.75</v>
+            <v>1403.55</v>
           </cell>
         </row>
         <row r="302">
@@ -9303,7 +9303,7 @@
             <v>2807.35</v>
           </cell>
           <cell r="BL302">
-            <v>3277.5</v>
+            <v>1867.65</v>
           </cell>
         </row>
         <row r="303">
@@ -9353,7 +9353,7 @@
             <v>153570.17000000001</v>
           </cell>
           <cell r="BL303">
-            <v>104267.16</v>
+            <v>80514.02</v>
           </cell>
         </row>
         <row r="304">
@@ -9403,7 +9403,7 @@
             <v>11988.76</v>
           </cell>
           <cell r="BL304">
-            <v>9025.65</v>
+            <v>6680.78</v>
           </cell>
         </row>
         <row r="305">
@@ -9453,7 +9453,7 @@
             <v>3782.99</v>
           </cell>
           <cell r="BL305">
-            <v>738.95</v>
+            <v>728.05</v>
           </cell>
         </row>
         <row r="306">
@@ -9503,7 +9503,7 @@
             <v>2317.5500000000002</v>
           </cell>
           <cell r="BL306">
-            <v>433</v>
+            <v>290</v>
           </cell>
         </row>
         <row r="307">
@@ -9553,7 +9553,7 @@
             <v>8450.7999999999993</v>
           </cell>
           <cell r="BL307">
-            <v>5317.21</v>
+            <v>3988.82</v>
           </cell>
         </row>
         <row r="308">
@@ -9603,7 +9603,7 @@
             <v>20216.419999999998</v>
           </cell>
           <cell r="BL308">
-            <v>29440.46</v>
+            <v>16613.75</v>
           </cell>
         </row>
         <row r="309">
@@ -9953,7 +9953,7 @@
             <v>5408.2</v>
           </cell>
           <cell r="BL317">
-            <v>6111.44</v>
+            <v>1786.26</v>
           </cell>
         </row>
         <row r="318">
@@ -10103,7 +10103,7 @@
             <v>2431.15</v>
           </cell>
           <cell r="BL320">
-            <v>6599.3</v>
+            <v>5449.8</v>
           </cell>
         </row>
         <row r="321">
@@ -10153,7 +10153,7 @@
             <v>2748.05</v>
           </cell>
           <cell r="BL321">
-            <v>4311.3900000000003</v>
+            <v>3777.22</v>
           </cell>
         </row>
         <row r="322">
@@ -10203,7 +10203,7 @@
             <v>5884.89</v>
           </cell>
           <cell r="BL322">
-            <v>3322.26</v>
+            <v>2263.23</v>
           </cell>
         </row>
         <row r="323">
@@ -10253,7 +10253,7 @@
             <v>5304.37</v>
           </cell>
           <cell r="BL323">
-            <v>11467.41</v>
+            <v>9542.5</v>
           </cell>
         </row>
         <row r="324">
@@ -10303,7 +10303,7 @@
             <v>630.75</v>
           </cell>
           <cell r="BL324">
-            <v>334.6</v>
+            <v>306.55</v>
           </cell>
         </row>
         <row r="325">
@@ -10403,7 +10403,7 @@
             <v>2586.27</v>
           </cell>
           <cell r="BL326">
-            <v>3023.3</v>
+            <v>2485.46</v>
           </cell>
         </row>
         <row r="327">
@@ -10453,7 +10453,7 @@
             <v>3384.9</v>
           </cell>
           <cell r="BL327">
-            <v>933.45</v>
+            <v>581.79999999999995</v>
           </cell>
         </row>
         <row r="328">
@@ -10503,7 +10503,7 @@
             <v>18556.27</v>
           </cell>
           <cell r="BL328">
-            <v>27058.66</v>
+            <v>21101.45</v>
           </cell>
         </row>
         <row r="329">
@@ -10553,7 +10553,7 @@
             <v>4790.9799999999996</v>
           </cell>
           <cell r="BL329">
-            <v>5364.02</v>
+            <v>4777.58</v>
           </cell>
         </row>
         <row r="330">
@@ -10603,7 +10603,7 @@
             <v>2022.35</v>
           </cell>
           <cell r="BL330">
-            <v>2293.94</v>
+            <v>1928.74</v>
           </cell>
         </row>
         <row r="331">
@@ -10703,7 +10703,7 @@
             <v>2024.05</v>
           </cell>
           <cell r="BL332">
-            <v>3385.8</v>
+            <v>2746.48</v>
           </cell>
         </row>
         <row r="333">
@@ -10753,7 +10753,7 @@
             <v>10644.94</v>
           </cell>
           <cell r="BL333">
-            <v>9179.16</v>
+            <v>7410.16</v>
           </cell>
         </row>
         <row r="334">
@@ -11103,7 +11103,7 @@
             <v>3516.16</v>
           </cell>
           <cell r="BL342">
-            <v>3672.38</v>
+            <v>2730.14</v>
           </cell>
         </row>
         <row r="343">
@@ -11253,7 +11253,7 @@
             <v>1706.35</v>
           </cell>
           <cell r="BL345">
-            <v>4098.6400000000003</v>
+            <v>3425.04</v>
           </cell>
         </row>
         <row r="346">
@@ -11303,7 +11303,7 @@
             <v>4351.96</v>
           </cell>
           <cell r="BL346">
-            <v>3043.23</v>
+            <v>2342.2600000000002</v>
           </cell>
         </row>
         <row r="347">
@@ -11353,7 +11353,7 @@
             <v>6772.9</v>
           </cell>
           <cell r="BL347">
-            <v>10696.59</v>
+            <v>9462.0300000000007</v>
           </cell>
         </row>
         <row r="348">
@@ -11403,7 +11403,7 @@
             <v>10251.93</v>
           </cell>
           <cell r="BL348">
-            <v>9913.24</v>
+            <v>8491.7800000000007</v>
           </cell>
         </row>
         <row r="349">
@@ -11453,7 +11453,7 @@
             <v>1478.26</v>
           </cell>
           <cell r="BL349">
-            <v>685.42</v>
+            <v>557.72</v>
           </cell>
         </row>
         <row r="350">
@@ -11553,7 +11553,7 @@
             <v>3188.47</v>
           </cell>
           <cell r="BL351">
-            <v>1029.7</v>
+            <v>740.1</v>
           </cell>
         </row>
         <row r="352">
@@ -11653,7 +11653,7 @@
             <v>29857.48</v>
           </cell>
           <cell r="BL353">
-            <v>25009.18</v>
+            <v>19624.55</v>
           </cell>
         </row>
         <row r="354">
@@ -11703,7 +11703,7 @@
             <v>6679.21</v>
           </cell>
           <cell r="BL354">
-            <v>5383.88</v>
+            <v>5071.66</v>
           </cell>
         </row>
         <row r="355">
@@ -11753,7 +11753,7 @@
             <v>3019.73</v>
           </cell>
           <cell r="BL355">
-            <v>1681.76</v>
+            <v>1557.26</v>
           </cell>
         </row>
         <row r="356">
@@ -11853,7 +11853,7 @@
             <v>4746.4399999999996</v>
           </cell>
           <cell r="BL357">
-            <v>4047.07</v>
+            <v>2570.84</v>
           </cell>
         </row>
         <row r="358">
@@ -11903,7 +11903,7 @@
             <v>18146.46</v>
           </cell>
           <cell r="BL358">
-            <v>21315.65</v>
+            <v>13052.18</v>
           </cell>
         </row>
         <row r="359">
@@ -13059,7 +13059,7 @@
         <v>109</v>
       </c>
       <c r="P4">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -13247,7 +13247,7 @@
         <v>108</v>
       </c>
       <c r="P5">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -13435,7 +13435,7 @@
         <v>277</v>
       </c>
       <c r="P6">
-        <v>177</v>
+        <v>116</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -13623,7 +13623,7 @@
         <v>5</v>
       </c>
       <c r="P7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -13811,7 +13811,7 @@
         <v>40</v>
       </c>
       <c r="P8">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -13999,7 +13999,7 @@
         <v>78</v>
       </c>
       <c r="P9">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="Q9">
         <v>0</v>
@@ -14375,7 +14375,7 @@
         <v>892</v>
       </c>
       <c r="P11">
-        <v>726</v>
+        <v>547</v>
       </c>
       <c r="Q11">
         <v>0</v>
@@ -14563,7 +14563,7 @@
         <v>425</v>
       </c>
       <c r="P12">
-        <v>508</v>
+        <v>390</v>
       </c>
       <c r="Q12">
         <v>0</v>
@@ -14751,7 +14751,7 @@
         <v>775</v>
       </c>
       <c r="P13">
-        <v>543</v>
+        <v>420</v>
       </c>
       <c r="Q13">
         <v>0</v>
@@ -15445,7 +15445,7 @@
         <v>0</v>
       </c>
       <c r="P22">
-        <v>1041.4000000000001</v>
+        <v>1047.4000000000001</v>
       </c>
       <c r="Q22">
         <v>0</v>
@@ -15522,7 +15522,7 @@
         <v>523.79</v>
       </c>
       <c r="P23">
-        <v>397.25</v>
+        <v>173.1</v>
       </c>
       <c r="Q23">
         <v>0</v>
@@ -15599,7 +15599,7 @@
         <v>599.47</v>
       </c>
       <c r="P24">
-        <v>530.91</v>
+        <v>537.89</v>
       </c>
       <c r="Q24">
         <v>0</v>
@@ -15753,7 +15753,7 @@
         <v>51.99</v>
       </c>
       <c r="P26">
-        <v>37.4</v>
+        <v>41.3</v>
       </c>
       <c r="Q26">
         <v>0</v>
@@ -16061,7 +16061,7 @@
         <v>1664.01</v>
       </c>
       <c r="P30">
-        <v>4848</v>
+        <v>217</v>
       </c>
       <c r="Q30">
         <v>0</v>
@@ -16138,7 +16138,7 @@
         <v>1644.31</v>
       </c>
       <c r="P31">
-        <v>2100.16</v>
+        <v>2027.17</v>
       </c>
       <c r="Q31">
         <v>0</v>
@@ -16369,7 +16369,7 @@
         <v>508.18</v>
       </c>
       <c r="P34">
-        <v>66.400000000000006</v>
+        <v>66.7</v>
       </c>
       <c r="Q34">
         <v>0</v>
@@ -16446,7 +16446,7 @@
         <v>548.19000000000005</v>
       </c>
       <c r="P35">
-        <v>737.05</v>
+        <v>114.6</v>
       </c>
       <c r="Q35">
         <v>0</v>
@@ -17370,7 +17370,7 @@
         <v>0</v>
       </c>
       <c r="P47">
-        <v>959.3</v>
+        <v>163</v>
       </c>
       <c r="Q47">
         <v>0</v>
@@ -17447,7 +17447,7 @@
         <v>423.9</v>
       </c>
       <c r="P48">
-        <v>619.61</v>
+        <v>579.05999999999995</v>
       </c>
       <c r="Q48">
         <v>0</v>
@@ -17524,7 +17524,7 @@
         <v>6771.6</v>
       </c>
       <c r="P49">
-        <v>994.28</v>
+        <v>907.53</v>
       </c>
       <c r="Q49">
         <v>0</v>
@@ -17601,7 +17601,7 @@
         <v>1756.31</v>
       </c>
       <c r="P50">
-        <v>507.14</v>
+        <v>441.39</v>
       </c>
       <c r="Q50">
         <v>0</v>
@@ -17678,7 +17678,7 @@
         <v>392.52</v>
       </c>
       <c r="P51">
-        <v>65.3</v>
+        <v>49.3</v>
       </c>
       <c r="Q51">
         <v>0</v>
@@ -17832,7 +17832,7 @@
         <v>475.55</v>
       </c>
       <c r="P53">
-        <v>51.64</v>
+        <v>29.94</v>
       </c>
       <c r="Q53">
         <v>0</v>
@@ -17986,7 +17986,7 @@
         <v>6968.14</v>
       </c>
       <c r="P55">
-        <v>743.18</v>
+        <v>731.48</v>
       </c>
       <c r="Q55">
         <v>0</v>
@@ -18063,7 +18063,7 @@
         <v>351.6</v>
       </c>
       <c r="P56">
-        <v>964.24</v>
+        <v>936.84</v>
       </c>
       <c r="Q56">
         <v>0</v>
@@ -18140,7 +18140,7 @@
         <v>275.2</v>
       </c>
       <c r="P57">
-        <v>334.8</v>
+        <v>281.3</v>
       </c>
       <c r="Q57">
         <v>0</v>
@@ -18294,7 +18294,7 @@
         <v>1453.89</v>
       </c>
       <c r="P59">
-        <v>632.67999999999995</v>
+        <v>492.81</v>
       </c>
       <c r="Q59">
         <v>0</v>
@@ -18371,7 +18371,7 @@
         <v>87.73</v>
       </c>
       <c r="P60">
-        <v>246.3</v>
+        <v>245.3</v>
       </c>
       <c r="Q60">
         <v>0</v>
@@ -19064,7 +19064,7 @@
         <v>1528.85</v>
       </c>
       <c r="P69">
-        <v>1436.72</v>
+        <v>1238.8</v>
       </c>
       <c r="Q69">
         <v>0</v>
@@ -19295,7 +19295,7 @@
         <v>806.7</v>
       </c>
       <c r="P72">
-        <v>699.1</v>
+        <v>579.29999999999995</v>
       </c>
       <c r="Q72">
         <v>0</v>
@@ -19372,7 +19372,7 @@
         <v>2564.08</v>
       </c>
       <c r="P73">
-        <v>923.53</v>
+        <v>331.3</v>
       </c>
       <c r="Q73">
         <v>0</v>
@@ -19449,7 +19449,7 @@
         <v>3205.26</v>
       </c>
       <c r="P74">
-        <v>1279.26</v>
+        <v>850.52</v>
       </c>
       <c r="Q74">
         <v>0</v>
@@ -19526,7 +19526,7 @@
         <v>5782.77</v>
       </c>
       <c r="P75">
-        <v>1377.73</v>
+        <v>882.29</v>
       </c>
       <c r="Q75">
         <v>0</v>
@@ -19603,7 +19603,7 @@
         <v>360.6</v>
       </c>
       <c r="P76">
-        <v>159.35</v>
+        <v>117.8</v>
       </c>
       <c r="Q76">
         <v>0</v>
@@ -19757,7 +19757,7 @@
         <v>276.93</v>
       </c>
       <c r="P78">
-        <v>215.83</v>
+        <v>150.47999999999999</v>
       </c>
       <c r="Q78">
         <v>0</v>
@@ -19911,7 +19911,7 @@
         <v>7670.07</v>
       </c>
       <c r="P80">
-        <v>4924.63</v>
+        <v>2479.83</v>
       </c>
       <c r="Q80">
         <v>0</v>
@@ -19988,7 +19988,7 @@
         <v>3574.39</v>
       </c>
       <c r="P81">
-        <v>2211.31</v>
+        <v>664.76</v>
       </c>
       <c r="Q81">
         <v>0</v>
@@ -20065,7 +20065,7 @@
         <v>799.37</v>
       </c>
       <c r="P82">
-        <v>586.82000000000005</v>
+        <v>552.47</v>
       </c>
       <c r="Q82">
         <v>0</v>
@@ -20219,7 +20219,7 @@
         <v>2160.71</v>
       </c>
       <c r="P84">
-        <v>2155.6799999999998</v>
+        <v>1177.83</v>
       </c>
       <c r="Q84">
         <v>0</v>
@@ -20296,7 +20296,7 @@
         <v>5356.76</v>
       </c>
       <c r="P85">
-        <v>2663.63</v>
+        <v>2421.7399999999998</v>
       </c>
       <c r="Q85">
         <v>0</v>
@@ -21374,7 +21374,7 @@
         <v>32.49</v>
       </c>
       <c r="P99">
-        <v>78.959999999999994</v>
+        <v>0.01</v>
       </c>
       <c r="Q99">
         <v>0</v>
@@ -21682,7 +21682,7 @@
         <v>0</v>
       </c>
       <c r="P103">
-        <v>5.56</v>
+        <v>0</v>
       </c>
       <c r="Q103">
         <v>0</v>
@@ -21913,7 +21913,7 @@
         <v>64.069999999999993</v>
       </c>
       <c r="P106">
-        <v>4.96</v>
+        <v>0</v>
       </c>
       <c r="Q106">
         <v>0</v>
@@ -23222,7 +23222,7 @@
         <v>203.03</v>
       </c>
       <c r="P123">
-        <v>21.49</v>
+        <v>17.89</v>
       </c>
       <c r="Q123">
         <v>0</v>
@@ -23376,7 +23376,7 @@
         <v>788.08</v>
       </c>
       <c r="P125">
-        <v>262.37</v>
+        <v>241.87</v>
       </c>
       <c r="Q125">
         <v>0</v>
@@ -23838,7 +23838,7 @@
         <v>128.09</v>
       </c>
       <c r="P131">
-        <v>460.75</v>
+        <v>466.05</v>
       </c>
       <c r="Q131">
         <v>0</v>
@@ -24069,7 +24069,7 @@
         <v>347.7</v>
       </c>
       <c r="P134">
-        <v>236.83</v>
+        <v>193.03</v>
       </c>
       <c r="Q134">
         <v>0</v>
@@ -25147,7 +25147,7 @@
         <v>449.41</v>
       </c>
       <c r="P148">
-        <v>493.17</v>
+        <v>436.87</v>
       </c>
       <c r="Q148">
         <v>0</v>
@@ -25224,7 +25224,7 @@
         <v>1131.74</v>
       </c>
       <c r="P149">
-        <v>354.19</v>
+        <v>304.58999999999997</v>
       </c>
       <c r="Q149">
         <v>0</v>
@@ -25301,7 +25301,7 @@
         <v>989.68</v>
       </c>
       <c r="P150">
-        <v>597.6</v>
+        <v>563.29999999999995</v>
       </c>
       <c r="Q150">
         <v>0</v>
@@ -25686,7 +25686,7 @@
         <v>1212.5</v>
       </c>
       <c r="P155">
-        <v>299.39999999999998</v>
+        <v>129.5</v>
       </c>
       <c r="Q155">
         <v>0</v>
@@ -25763,7 +25763,7 @@
         <v>1217.27</v>
       </c>
       <c r="P156">
-        <v>213.08</v>
+        <v>199.18</v>
       </c>
       <c r="Q156">
         <v>0</v>
@@ -25994,7 +25994,7 @@
         <v>332.2</v>
       </c>
       <c r="P159">
-        <v>482.65</v>
+        <v>470.95</v>
       </c>
       <c r="Q159">
         <v>0</v>
@@ -26071,7 +26071,7 @@
         <v>282.8</v>
       </c>
       <c r="P160">
-        <v>585.54999999999995</v>
+        <v>313.75</v>
       </c>
       <c r="Q160">
         <v>0</v>
@@ -28689,7 +28689,7 @@
         <v>10911.5</v>
       </c>
       <c r="P194">
-        <v>21505.040000000001</v>
+        <v>7867.21</v>
       </c>
       <c r="Q194">
         <v>0</v>
@@ -28920,7 +28920,7 @@
         <v>9643.9500000000007</v>
       </c>
       <c r="P197">
-        <v>5286.1</v>
+        <v>4716.7</v>
       </c>
       <c r="Q197">
         <v>0</v>
@@ -28997,7 +28997,7 @@
         <v>7099.57</v>
       </c>
       <c r="P198">
-        <v>9589.81</v>
+        <v>5330.29</v>
       </c>
       <c r="Q198">
         <v>0</v>
@@ -29074,7 +29074,7 @@
         <v>10437.030000000001</v>
       </c>
       <c r="P199">
-        <v>9748.14</v>
+        <v>8063.34</v>
       </c>
       <c r="Q199">
         <v>0</v>
@@ -29151,7 +29151,7 @@
         <v>14032.28</v>
       </c>
       <c r="P200">
-        <v>15233.71</v>
+        <v>10665.79</v>
       </c>
       <c r="Q200">
         <v>0</v>
@@ -29228,7 +29228,7 @@
         <v>819.93</v>
       </c>
       <c r="P201">
-        <v>1123.31</v>
+        <v>649.42999999999995</v>
       </c>
       <c r="Q201">
         <v>0</v>
@@ -29382,7 +29382,7 @@
         <v>1498.34</v>
       </c>
       <c r="P203">
-        <v>2654.75</v>
+        <v>1403.55</v>
       </c>
       <c r="Q203">
         <v>0</v>
@@ -29459,7 +29459,7 @@
         <v>2807.35</v>
       </c>
       <c r="P204">
-        <v>3277.5</v>
+        <v>1867.65</v>
       </c>
       <c r="Q204">
         <v>0</v>
@@ -29536,7 +29536,7 @@
         <v>153570.17000000001</v>
       </c>
       <c r="P205">
-        <v>104267.16</v>
+        <v>80514.02</v>
       </c>
       <c r="Q205">
         <v>0</v>
@@ -29613,7 +29613,7 @@
         <v>11988.76</v>
       </c>
       <c r="P206">
-        <v>9025.65</v>
+        <v>6680.78</v>
       </c>
       <c r="Q206">
         <v>0</v>
@@ -29690,7 +29690,7 @@
         <v>3782.99</v>
       </c>
       <c r="P207">
-        <v>738.95</v>
+        <v>728.05</v>
       </c>
       <c r="Q207">
         <v>0</v>
@@ -29767,7 +29767,7 @@
         <v>2317.5500000000002</v>
       </c>
       <c r="P208">
-        <v>433</v>
+        <v>290</v>
       </c>
       <c r="Q208">
         <v>0</v>
@@ -29844,7 +29844,7 @@
         <v>8450.7999999999993</v>
       </c>
       <c r="P209">
-        <v>5317.21</v>
+        <v>3988.82</v>
       </c>
       <c r="Q209">
         <v>0</v>
@@ -29921,7 +29921,7 @@
         <v>20216.419999999998</v>
       </c>
       <c r="P210">
-        <v>29440.46</v>
+        <v>16613.75</v>
       </c>
       <c r="Q210">
         <v>0</v>
@@ -30614,7 +30614,7 @@
         <v>5408.2</v>
       </c>
       <c r="P219">
-        <v>6111.44</v>
+        <v>1786.26</v>
       </c>
       <c r="Q219">
         <v>0</v>
@@ -30845,7 +30845,7 @@
         <v>2431.15</v>
       </c>
       <c r="P222">
-        <v>6599.3</v>
+        <v>5449.8</v>
       </c>
       <c r="Q222">
         <v>0</v>
@@ -30922,7 +30922,7 @@
         <v>2748.05</v>
       </c>
       <c r="P223">
-        <v>4311.3900000000003</v>
+        <v>3777.22</v>
       </c>
       <c r="Q223">
         <v>0</v>
@@ -30999,7 +30999,7 @@
         <v>5884.89</v>
       </c>
       <c r="P224">
-        <v>3322.26</v>
+        <v>2263.23</v>
       </c>
       <c r="Q224">
         <v>0</v>
@@ -31076,7 +31076,7 @@
         <v>5304.37</v>
       </c>
       <c r="P225">
-        <v>11467.41</v>
+        <v>9542.5</v>
       </c>
       <c r="Q225">
         <v>0</v>
@@ -31153,7 +31153,7 @@
         <v>630.75</v>
       </c>
       <c r="P226">
-        <v>334.6</v>
+        <v>306.55</v>
       </c>
       <c r="Q226">
         <v>0</v>
@@ -31307,7 +31307,7 @@
         <v>2586.27</v>
       </c>
       <c r="P228">
-        <v>3023.3</v>
+        <v>2485.46</v>
       </c>
       <c r="Q228">
         <v>0</v>
@@ -31384,7 +31384,7 @@
         <v>3384.9</v>
       </c>
       <c r="P229">
-        <v>933.45</v>
+        <v>581.79999999999995</v>
       </c>
       <c r="Q229">
         <v>0</v>
@@ -31461,7 +31461,7 @@
         <v>18556.27</v>
       </c>
       <c r="P230">
-        <v>27058.66</v>
+        <v>21101.45</v>
       </c>
       <c r="Q230">
         <v>0</v>
@@ -31538,7 +31538,7 @@
         <v>4790.9799999999996</v>
       </c>
       <c r="P231">
-        <v>5364.02</v>
+        <v>4777.58</v>
       </c>
       <c r="Q231">
         <v>0</v>
@@ -31615,7 +31615,7 @@
         <v>2022.35</v>
       </c>
       <c r="P232">
-        <v>2293.94</v>
+        <v>1928.74</v>
       </c>
       <c r="Q232">
         <v>0</v>
@@ -31769,7 +31769,7 @@
         <v>2024.05</v>
       </c>
       <c r="P234">
-        <v>3385.8</v>
+        <v>2746.48</v>
       </c>
       <c r="Q234">
         <v>0</v>
@@ -31846,7 +31846,7 @@
         <v>10644.94</v>
       </c>
       <c r="P235">
-        <v>9179.16</v>
+        <v>7410.16</v>
       </c>
       <c r="Q235">
         <v>0</v>
@@ -32539,7 +32539,7 @@
         <v>3516.16</v>
       </c>
       <c r="P244">
-        <v>3672.38</v>
+        <v>2730.14</v>
       </c>
       <c r="Q244">
         <v>0</v>
@@ -32770,7 +32770,7 @@
         <v>1706.35</v>
       </c>
       <c r="P247">
-        <v>4098.6400000000003</v>
+        <v>3425.04</v>
       </c>
       <c r="Q247">
         <v>0</v>
@@ -32847,7 +32847,7 @@
         <v>4351.96</v>
       </c>
       <c r="P248">
-        <v>3043.23</v>
+        <v>2342.2600000000002</v>
       </c>
       <c r="Q248">
         <v>0</v>
@@ -32924,7 +32924,7 @@
         <v>6772.9</v>
       </c>
       <c r="P249">
-        <v>10696.59</v>
+        <v>9462.0300000000007</v>
       </c>
       <c r="Q249">
         <v>0</v>
@@ -33001,7 +33001,7 @@
         <v>10251.93</v>
       </c>
       <c r="P250">
-        <v>9913.24</v>
+        <v>8491.7800000000007</v>
       </c>
       <c r="Q250">
         <v>0</v>
@@ -33078,7 +33078,7 @@
         <v>1478.26</v>
       </c>
       <c r="P251">
-        <v>685.42</v>
+        <v>557.72</v>
       </c>
       <c r="Q251">
         <v>0</v>
@@ -33232,7 +33232,7 @@
         <v>3188.47</v>
       </c>
       <c r="P253">
-        <v>1029.7</v>
+        <v>740.1</v>
       </c>
       <c r="Q253">
         <v>0</v>
@@ -33386,7 +33386,7 @@
         <v>29857.48</v>
       </c>
       <c r="P255">
-        <v>25009.18</v>
+        <v>19624.55</v>
       </c>
       <c r="Q255">
         <v>0</v>
@@ -33463,7 +33463,7 @@
         <v>6679.21</v>
       </c>
       <c r="P256">
-        <v>5383.88</v>
+        <v>5071.66</v>
       </c>
       <c r="Q256">
         <v>0</v>
@@ -33540,7 +33540,7 @@
         <v>3019.73</v>
       </c>
       <c r="P257">
-        <v>1681.76</v>
+        <v>1557.26</v>
       </c>
       <c r="Q257">
         <v>0</v>
@@ -33694,7 +33694,7 @@
         <v>4746.4399999999996</v>
       </c>
       <c r="P259">
-        <v>4047.07</v>
+        <v>2570.84</v>
       </c>
       <c r="Q259">
         <v>0</v>
@@ -33771,7 +33771,7 @@
         <v>18146.46</v>
       </c>
       <c r="P260">
-        <v>21315.65</v>
+        <v>13052.18</v>
       </c>
       <c r="Q260">
         <v>0</v>

</xml_diff>

<commit_message>
fix: atualiza app.py e vendas.xlsx
</commit_message>
<xml_diff>
--- a/vendas.xlsx
+++ b/vendas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/60bd3766fe3b56c0/Nova pasta/Nova pasta/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Claudio\Documents\verdent-projects\new-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2C66AA5-2F67-4010-B837-35B29476A991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948D37CA-6BA6-4568-ACB2-341A1391D80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F2DED76B-5FEA-48D5-9DAC-66F60A430568}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Qtd. vendas por funcionário</t>
   </si>
@@ -104,6 +104,9 @@
   <si>
     <t xml:space="preserve">vendas por setores </t>
   </si>
+  <si>
+    <t xml:space="preserve">TOTAL ENTRADA </t>
+  </si>
 </sst>
 </file>
 
@@ -111,7 +114,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="7" formatCode="&quot;R$&quot;\ #,##0.00;\-&quot;R$&quot;\ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="mmmm\,\ yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="mmmm\,\ yyyy;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -144,7 +147,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -246,7 +249,7 @@
             <v>109</v>
           </cell>
           <cell r="BL93">
-            <v>54</v>
+            <v>67</v>
           </cell>
         </row>
         <row r="94">
@@ -290,7 +293,7 @@
             <v>108</v>
           </cell>
           <cell r="BL94">
-            <v>68</v>
+            <v>91</v>
           </cell>
         </row>
         <row r="95">
@@ -334,7 +337,7 @@
             <v>277</v>
           </cell>
           <cell r="BL95">
-            <v>116</v>
+            <v>185</v>
           </cell>
         </row>
         <row r="96">
@@ -378,7 +381,7 @@
             <v>5</v>
           </cell>
           <cell r="BL96">
-            <v>4</v>
+            <v>6</v>
           </cell>
         </row>
         <row r="97">
@@ -422,7 +425,7 @@
             <v>40</v>
           </cell>
           <cell r="BL97">
-            <v>28</v>
+            <v>36</v>
           </cell>
         </row>
         <row r="98">
@@ -466,7 +469,7 @@
             <v>78</v>
           </cell>
           <cell r="BL98">
-            <v>57</v>
+            <v>70</v>
           </cell>
         </row>
         <row r="99">
@@ -554,7 +557,7 @@
             <v>892</v>
           </cell>
           <cell r="BL100">
-            <v>547</v>
+            <v>751</v>
           </cell>
         </row>
         <row r="101">
@@ -598,7 +601,7 @@
             <v>425</v>
           </cell>
           <cell r="BL101">
-            <v>390</v>
+            <v>561</v>
           </cell>
         </row>
         <row r="102">
@@ -642,7 +645,7 @@
             <v>775</v>
           </cell>
           <cell r="BL102">
-            <v>420</v>
+            <v>588</v>
           </cell>
         </row>
         <row r="103">
@@ -903,7 +906,7 @@
             <v>0</v>
           </cell>
           <cell r="BL120">
-            <v>1047.4000000000001</v>
+            <v>1041.4000000000001</v>
           </cell>
         </row>
         <row r="121">
@@ -953,7 +956,7 @@
             <v>523.79</v>
           </cell>
           <cell r="BL121">
-            <v>173.1</v>
+            <v>444.05</v>
           </cell>
         </row>
         <row r="122">
@@ -1003,7 +1006,7 @@
             <v>599.47</v>
           </cell>
           <cell r="BL122">
-            <v>537.89</v>
+            <v>545.91</v>
           </cell>
         </row>
         <row r="123">
@@ -1053,7 +1056,7 @@
             <v>963.68</v>
           </cell>
           <cell r="BL123">
-            <v>421.07</v>
+            <v>580.96</v>
           </cell>
         </row>
         <row r="124">
@@ -1103,7 +1106,7 @@
             <v>51.99</v>
           </cell>
           <cell r="BL124">
-            <v>41.3</v>
+            <v>37.4</v>
           </cell>
         </row>
         <row r="125">
@@ -1203,7 +1206,7 @@
             <v>213.94</v>
           </cell>
           <cell r="BL126">
-            <v>86</v>
+            <v>95.9</v>
           </cell>
         </row>
         <row r="127">
@@ -1303,7 +1306,7 @@
             <v>1664.01</v>
           </cell>
           <cell r="BL128">
-            <v>217</v>
+            <v>4848</v>
           </cell>
         </row>
         <row r="129">
@@ -1353,7 +1356,7 @@
             <v>1644.31</v>
           </cell>
           <cell r="BL129">
-            <v>2027.17</v>
+            <v>2100.16</v>
           </cell>
         </row>
         <row r="130">
@@ -1403,7 +1406,7 @@
             <v>251.68</v>
           </cell>
           <cell r="BL130">
-            <v>517.14</v>
+            <v>530.04</v>
           </cell>
         </row>
         <row r="131">
@@ -1503,7 +1506,7 @@
             <v>508.18</v>
           </cell>
           <cell r="BL132">
-            <v>66.7</v>
+            <v>86.4</v>
           </cell>
         </row>
         <row r="133">
@@ -1553,7 +1556,7 @@
             <v>548.19000000000005</v>
           </cell>
           <cell r="BL133">
-            <v>114.6</v>
+            <v>758.05</v>
           </cell>
         </row>
         <row r="134">
@@ -2053,7 +2056,7 @@
             <v>0</v>
           </cell>
           <cell r="BL145">
-            <v>163</v>
+            <v>959.3</v>
           </cell>
         </row>
         <row r="146">
@@ -2103,7 +2106,7 @@
             <v>423.9</v>
           </cell>
           <cell r="BL146">
-            <v>579.05999999999995</v>
+            <v>619.61</v>
           </cell>
         </row>
         <row r="147">
@@ -2153,7 +2156,7 @@
             <v>6771.6</v>
           </cell>
           <cell r="BL147">
-            <v>907.53</v>
+            <v>991.28</v>
           </cell>
         </row>
         <row r="148">
@@ -2203,7 +2206,7 @@
             <v>1756.31</v>
           </cell>
           <cell r="BL148">
-            <v>441.39</v>
+            <v>505.85</v>
           </cell>
         </row>
         <row r="149">
@@ -2253,7 +2256,7 @@
             <v>392.52</v>
           </cell>
           <cell r="BL149">
-            <v>49.3</v>
+            <v>65.3</v>
           </cell>
         </row>
         <row r="150">
@@ -2353,7 +2356,7 @@
             <v>475.55</v>
           </cell>
           <cell r="BL151">
-            <v>29.94</v>
+            <v>74.64</v>
           </cell>
         </row>
         <row r="152">
@@ -2453,7 +2456,7 @@
             <v>6968.14</v>
           </cell>
           <cell r="BL153">
-            <v>731.48</v>
+            <v>743.18</v>
           </cell>
         </row>
         <row r="154">
@@ -2503,7 +2506,7 @@
             <v>351.6</v>
           </cell>
           <cell r="BL154">
-            <v>936.84</v>
+            <v>1244.1199999999999</v>
           </cell>
         </row>
         <row r="155">
@@ -2553,7 +2556,7 @@
             <v>275.2</v>
           </cell>
           <cell r="BL155">
-            <v>281.3</v>
+            <v>334.8</v>
           </cell>
         </row>
         <row r="156">
@@ -2653,7 +2656,7 @@
             <v>1453.89</v>
           </cell>
           <cell r="BL157">
-            <v>492.81</v>
+            <v>667.68</v>
           </cell>
         </row>
         <row r="158">
@@ -2703,7 +2706,7 @@
             <v>87.73</v>
           </cell>
           <cell r="BL158">
-            <v>245.3</v>
+            <v>266.25</v>
           </cell>
         </row>
         <row r="159">
@@ -3053,7 +3056,7 @@
             <v>1528.85</v>
           </cell>
           <cell r="BL167">
-            <v>1238.8</v>
+            <v>2994.32</v>
           </cell>
         </row>
         <row r="168">
@@ -3203,7 +3206,7 @@
             <v>806.7</v>
           </cell>
           <cell r="BL170">
-            <v>579.29999999999995</v>
+            <v>699.1</v>
           </cell>
         </row>
         <row r="171">
@@ -3253,7 +3256,7 @@
             <v>2564.08</v>
           </cell>
           <cell r="BL171">
-            <v>331.3</v>
+            <v>946.13</v>
           </cell>
         </row>
         <row r="172">
@@ -3303,7 +3306,7 @@
             <v>3205.26</v>
           </cell>
           <cell r="BL172">
-            <v>850.52</v>
+            <v>1296.3599999999999</v>
           </cell>
         </row>
         <row r="173">
@@ -3353,7 +3356,7 @@
             <v>5782.77</v>
           </cell>
           <cell r="BL173">
-            <v>882.29</v>
+            <v>1352.67</v>
           </cell>
         </row>
         <row r="174">
@@ -3403,7 +3406,7 @@
             <v>360.6</v>
           </cell>
           <cell r="BL174">
-            <v>117.8</v>
+            <v>163.25</v>
           </cell>
         </row>
         <row r="175">
@@ -3503,7 +3506,7 @@
             <v>276.93</v>
           </cell>
           <cell r="BL176">
-            <v>150.47999999999999</v>
+            <v>209.83</v>
           </cell>
         </row>
         <row r="177">
@@ -3603,7 +3606,7 @@
             <v>7670.07</v>
           </cell>
           <cell r="BL178">
-            <v>2479.83</v>
+            <v>4804.8999999999996</v>
           </cell>
         </row>
         <row r="179">
@@ -3653,7 +3656,7 @@
             <v>3574.39</v>
           </cell>
           <cell r="BL179">
-            <v>664.76</v>
+            <v>2210.5100000000002</v>
           </cell>
         </row>
         <row r="180">
@@ -3703,7 +3706,7 @@
             <v>799.37</v>
           </cell>
           <cell r="BL180">
-            <v>552.47</v>
+            <v>603.72</v>
           </cell>
         </row>
         <row r="181">
@@ -3803,7 +3806,7 @@
             <v>2160.71</v>
           </cell>
           <cell r="BL182">
-            <v>1177.83</v>
+            <v>2207.09</v>
           </cell>
         </row>
         <row r="183">
@@ -3853,7 +3856,7 @@
             <v>5356.76</v>
           </cell>
           <cell r="BL183">
-            <v>2421.7399999999998</v>
+            <v>3423.97</v>
           </cell>
         </row>
         <row r="184">
@@ -4453,7 +4456,7 @@
             <v>32.49</v>
           </cell>
           <cell r="BL197">
-            <v>0.01</v>
+            <v>78.959999999999994</v>
           </cell>
         </row>
         <row r="198">
@@ -4653,7 +4656,7 @@
             <v>0</v>
           </cell>
           <cell r="BL201">
-            <v>0</v>
+            <v>5.56</v>
           </cell>
         </row>
         <row r="202">
@@ -4803,7 +4806,7 @@
             <v>64.069999999999993</v>
           </cell>
           <cell r="BL204">
-            <v>0</v>
+            <v>4.96</v>
           </cell>
         </row>
         <row r="205">
@@ -5553,7 +5556,7 @@
             <v>203.03</v>
           </cell>
           <cell r="BL221">
-            <v>17.89</v>
+            <v>21.49</v>
           </cell>
         </row>
         <row r="222">
@@ -5603,7 +5606,7 @@
             <v>540.03</v>
           </cell>
           <cell r="BL222">
-            <v>207.8</v>
+            <v>215.71</v>
           </cell>
         </row>
         <row r="223">
@@ -5653,7 +5656,7 @@
             <v>788.08</v>
           </cell>
           <cell r="BL223">
-            <v>241.87</v>
+            <v>253.37</v>
           </cell>
         </row>
         <row r="224">
@@ -5703,7 +5706,7 @@
             <v>349.1</v>
           </cell>
           <cell r="BL224">
-            <v>224.6</v>
+            <v>251.5</v>
           </cell>
         </row>
         <row r="225">
@@ -5953,7 +5956,7 @@
             <v>128.09</v>
           </cell>
           <cell r="BL229">
-            <v>466.05</v>
+            <v>572.65</v>
           </cell>
         </row>
         <row r="230">
@@ -6103,7 +6106,7 @@
             <v>347.7</v>
           </cell>
           <cell r="BL232">
-            <v>193.03</v>
+            <v>234.83</v>
           </cell>
         </row>
         <row r="233">
@@ -6703,7 +6706,7 @@
             <v>449.41</v>
           </cell>
           <cell r="BL246">
-            <v>436.87</v>
+            <v>482.17</v>
           </cell>
         </row>
         <row r="247">
@@ -6753,7 +6756,7 @@
             <v>1131.74</v>
           </cell>
           <cell r="BL247">
-            <v>304.58999999999997</v>
+            <v>347.79</v>
           </cell>
         </row>
         <row r="248">
@@ -6803,7 +6806,7 @@
             <v>989.68</v>
           </cell>
           <cell r="BL248">
-            <v>563.29999999999995</v>
+            <v>593.75</v>
           </cell>
         </row>
         <row r="249">
@@ -7053,7 +7056,7 @@
             <v>1212.5</v>
           </cell>
           <cell r="BL253">
-            <v>129.5</v>
+            <v>299.39999999999998</v>
           </cell>
         </row>
         <row r="254">
@@ -7103,7 +7106,7 @@
             <v>1217.27</v>
           </cell>
           <cell r="BL254">
-            <v>199.18</v>
+            <v>213.08</v>
           </cell>
         </row>
         <row r="255">
@@ -7253,7 +7256,7 @@
             <v>332.2</v>
           </cell>
           <cell r="BL257">
-            <v>470.95</v>
+            <v>482.65</v>
           </cell>
         </row>
         <row r="258">
@@ -7303,7 +7306,7 @@
             <v>282.8</v>
           </cell>
           <cell r="BL258">
-            <v>313.75</v>
+            <v>576.54999999999995</v>
           </cell>
         </row>
         <row r="259">
@@ -8803,7 +8806,7 @@
             <v>10911.5</v>
           </cell>
           <cell r="BL292">
-            <v>7867.21</v>
+            <v>24876.79</v>
           </cell>
         </row>
         <row r="293">
@@ -8953,7 +8956,7 @@
             <v>9643.9500000000007</v>
           </cell>
           <cell r="BL295">
-            <v>4716.7</v>
+            <v>5779.94</v>
           </cell>
         </row>
         <row r="296">
@@ -9003,7 +9006,7 @@
             <v>7099.57</v>
           </cell>
           <cell r="BL296">
-            <v>5330.29</v>
+            <v>9705.77</v>
           </cell>
         </row>
         <row r="297">
@@ -9053,7 +9056,7 @@
             <v>10437.030000000001</v>
           </cell>
           <cell r="BL297">
-            <v>8063.34</v>
+            <v>9755.67</v>
           </cell>
         </row>
         <row r="298">
@@ -9103,7 +9106,7 @@
             <v>14032.28</v>
           </cell>
           <cell r="BL298">
-            <v>10665.79</v>
+            <v>15322.7</v>
           </cell>
         </row>
         <row r="299">
@@ -9153,7 +9156,7 @@
             <v>819.93</v>
           </cell>
           <cell r="BL299">
-            <v>649.42999999999995</v>
+            <v>1161.1600000000001</v>
           </cell>
         </row>
         <row r="300">
@@ -9253,7 +9256,7 @@
             <v>1498.34</v>
           </cell>
           <cell r="BL301">
-            <v>1403.55</v>
+            <v>5223.99</v>
           </cell>
         </row>
         <row r="302">
@@ -9303,7 +9306,7 @@
             <v>2807.35</v>
           </cell>
           <cell r="BL302">
-            <v>1867.65</v>
+            <v>3277.5</v>
           </cell>
         </row>
         <row r="303">
@@ -9353,7 +9356,7 @@
             <v>153570.17000000001</v>
           </cell>
           <cell r="BL303">
-            <v>80514.02</v>
+            <v>109524.39</v>
           </cell>
         </row>
         <row r="304">
@@ -9403,7 +9406,7 @@
             <v>11988.76</v>
           </cell>
           <cell r="BL304">
-            <v>6680.78</v>
+            <v>9043.35</v>
           </cell>
         </row>
         <row r="305">
@@ -9453,7 +9456,7 @@
             <v>3782.99</v>
           </cell>
           <cell r="BL305">
-            <v>728.05</v>
+            <v>783.75</v>
           </cell>
         </row>
         <row r="306">
@@ -9503,7 +9506,7 @@
             <v>2317.5500000000002</v>
           </cell>
           <cell r="BL306">
-            <v>290</v>
+            <v>433</v>
           </cell>
         </row>
         <row r="307">
@@ -9553,7 +9556,7 @@
             <v>8450.7999999999993</v>
           </cell>
           <cell r="BL307">
-            <v>3988.82</v>
+            <v>5353.31</v>
           </cell>
         </row>
         <row r="308">
@@ -9603,7 +9606,7 @@
             <v>20216.419999999998</v>
           </cell>
           <cell r="BL308">
-            <v>16613.75</v>
+            <v>29217.46</v>
           </cell>
         </row>
         <row r="309">
@@ -9953,7 +9956,7 @@
             <v>5408.2</v>
           </cell>
           <cell r="BL317">
-            <v>1786.26</v>
+            <v>6246.19</v>
           </cell>
         </row>
         <row r="318">
@@ -10103,7 +10106,7 @@
             <v>2431.15</v>
           </cell>
           <cell r="BL320">
-            <v>5449.8</v>
+            <v>6642.2</v>
           </cell>
         </row>
         <row r="321">
@@ -10153,7 +10156,7 @@
             <v>2748.05</v>
           </cell>
           <cell r="BL321">
-            <v>3777.22</v>
+            <v>4725.95</v>
           </cell>
         </row>
         <row r="322">
@@ -10203,7 +10206,7 @@
             <v>5884.89</v>
           </cell>
           <cell r="BL322">
-            <v>2263.23</v>
+            <v>3883.83</v>
           </cell>
         </row>
         <row r="323">
@@ -10253,7 +10256,7 @@
             <v>5304.37</v>
           </cell>
           <cell r="BL323">
-            <v>9542.5</v>
+            <v>12189.58</v>
           </cell>
         </row>
         <row r="324">
@@ -10303,7 +10306,7 @@
             <v>630.75</v>
           </cell>
           <cell r="BL324">
-            <v>306.55</v>
+            <v>401.36</v>
           </cell>
         </row>
         <row r="325">
@@ -10403,7 +10406,7 @@
             <v>2586.27</v>
           </cell>
           <cell r="BL326">
-            <v>2485.46</v>
+            <v>3183.25</v>
           </cell>
         </row>
         <row r="327">
@@ -10453,7 +10456,7 @@
             <v>3384.9</v>
           </cell>
           <cell r="BL327">
-            <v>581.79999999999995</v>
+            <v>933.45</v>
           </cell>
         </row>
         <row r="328">
@@ -10503,7 +10506,7 @@
             <v>18556.27</v>
           </cell>
           <cell r="BL328">
-            <v>21101.45</v>
+            <v>32367.51</v>
           </cell>
         </row>
         <row r="329">
@@ -10553,7 +10556,7 @@
             <v>4790.9799999999996</v>
           </cell>
           <cell r="BL329">
-            <v>4777.58</v>
+            <v>5632.88</v>
           </cell>
         </row>
         <row r="330">
@@ -10603,7 +10606,7 @@
             <v>2022.35</v>
           </cell>
           <cell r="BL330">
-            <v>1928.74</v>
+            <v>2400.84</v>
           </cell>
         </row>
         <row r="331">
@@ -10703,7 +10706,7 @@
             <v>2024.05</v>
           </cell>
           <cell r="BL332">
-            <v>2746.48</v>
+            <v>3953.57</v>
           </cell>
         </row>
         <row r="333">
@@ -10753,7 +10756,7 @@
             <v>10644.94</v>
           </cell>
           <cell r="BL333">
-            <v>7410.16</v>
+            <v>9696.7800000000007</v>
           </cell>
         </row>
         <row r="334">
@@ -11103,7 +11106,7 @@
             <v>3516.16</v>
           </cell>
           <cell r="BL342">
-            <v>2730.14</v>
+            <v>4491.96</v>
           </cell>
         </row>
         <row r="343">
@@ -11253,7 +11256,7 @@
             <v>1706.35</v>
           </cell>
           <cell r="BL345">
-            <v>3425.04</v>
+            <v>4092.26</v>
           </cell>
         </row>
         <row r="346">
@@ -11303,7 +11306,7 @@
             <v>4351.96</v>
           </cell>
           <cell r="BL346">
-            <v>2342.2600000000002</v>
+            <v>3180.69</v>
           </cell>
         </row>
         <row r="347">
@@ -11353,7 +11356,7 @@
             <v>6772.9</v>
           </cell>
           <cell r="BL347">
-            <v>9462.0300000000007</v>
+            <v>10828.19</v>
           </cell>
         </row>
         <row r="348">
@@ -11403,7 +11406,7 @@
             <v>10251.93</v>
           </cell>
           <cell r="BL348">
-            <v>8491.7800000000007</v>
+            <v>10434.879999999999</v>
           </cell>
         </row>
         <row r="349">
@@ -11453,7 +11456,7 @@
             <v>1478.26</v>
           </cell>
           <cell r="BL349">
-            <v>557.72</v>
+            <v>716.95</v>
           </cell>
         </row>
         <row r="350">
@@ -11553,7 +11556,7 @@
             <v>3188.47</v>
           </cell>
           <cell r="BL351">
-            <v>740.1</v>
+            <v>1438.9</v>
           </cell>
         </row>
         <row r="352">
@@ -11653,7 +11656,7 @@
             <v>29857.48</v>
           </cell>
           <cell r="BL353">
-            <v>19624.55</v>
+            <v>26068.95</v>
           </cell>
         </row>
         <row r="354">
@@ -11703,7 +11706,7 @@
             <v>6679.21</v>
           </cell>
           <cell r="BL354">
-            <v>5071.66</v>
+            <v>5420.08</v>
           </cell>
         </row>
         <row r="355">
@@ -11753,7 +11756,7 @@
             <v>3019.73</v>
           </cell>
           <cell r="BL355">
-            <v>1557.26</v>
+            <v>1691.66</v>
           </cell>
         </row>
         <row r="356">
@@ -11853,7 +11856,7 @@
             <v>4746.4399999999996</v>
           </cell>
           <cell r="BL357">
-            <v>2570.84</v>
+            <v>4220.72</v>
           </cell>
         </row>
         <row r="358">
@@ -11903,7 +11906,7 @@
             <v>18146.46</v>
           </cell>
           <cell r="BL358">
-            <v>13052.18</v>
+            <v>22736.11</v>
           </cell>
         </row>
         <row r="359">
@@ -12901,7 +12904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A45DA6-73B0-4E2B-A1BA-FBFE1A2F5414}">
-  <dimension ref="A1:BK292"/>
+  <dimension ref="A1:BK299"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.42578125" customWidth="1"/>
@@ -13059,7 +13062,7 @@
         <v>109</v>
       </c>
       <c r="P4">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -13247,7 +13250,7 @@
         <v>108</v>
       </c>
       <c r="P5">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -13435,7 +13438,7 @@
         <v>277</v>
       </c>
       <c r="P6">
-        <v>116</v>
+        <v>185</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -13623,7 +13626,7 @@
         <v>5</v>
       </c>
       <c r="P7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -13811,7 +13814,7 @@
         <v>40</v>
       </c>
       <c r="P8">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -13999,7 +14002,7 @@
         <v>78</v>
       </c>
       <c r="P9">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="Q9">
         <v>0</v>
@@ -14375,7 +14378,7 @@
         <v>892</v>
       </c>
       <c r="P11">
-        <v>547</v>
+        <v>751</v>
       </c>
       <c r="Q11">
         <v>0</v>
@@ -14563,7 +14566,7 @@
         <v>425</v>
       </c>
       <c r="P12">
-        <v>390</v>
+        <v>561</v>
       </c>
       <c r="Q12">
         <v>0</v>
@@ -14751,7 +14754,7 @@
         <v>775</v>
       </c>
       <c r="P13">
-        <v>420</v>
+        <v>588</v>
       </c>
       <c r="Q13">
         <v>0</v>
@@ -15445,7 +15448,7 @@
         <v>0</v>
       </c>
       <c r="P22">
-        <v>1047.4000000000001</v>
+        <v>1041.4000000000001</v>
       </c>
       <c r="Q22">
         <v>0</v>
@@ -15522,7 +15525,7 @@
         <v>523.79</v>
       </c>
       <c r="P23">
-        <v>173.1</v>
+        <v>444.05</v>
       </c>
       <c r="Q23">
         <v>0</v>
@@ -15599,7 +15602,7 @@
         <v>599.47</v>
       </c>
       <c r="P24">
-        <v>537.89</v>
+        <v>545.91</v>
       </c>
       <c r="Q24">
         <v>0</v>
@@ -15676,7 +15679,7 @@
         <v>963.68</v>
       </c>
       <c r="P25">
-        <v>421.07</v>
+        <v>580.96</v>
       </c>
       <c r="Q25">
         <v>0</v>
@@ -15753,7 +15756,7 @@
         <v>51.99</v>
       </c>
       <c r="P26">
-        <v>41.3</v>
+        <v>37.4</v>
       </c>
       <c r="Q26">
         <v>0</v>
@@ -15907,7 +15910,7 @@
         <v>213.94</v>
       </c>
       <c r="P28">
-        <v>86</v>
+        <v>95.9</v>
       </c>
       <c r="Q28">
         <v>0</v>
@@ -16061,7 +16064,7 @@
         <v>1664.01</v>
       </c>
       <c r="P30">
-        <v>217</v>
+        <v>4848</v>
       </c>
       <c r="Q30">
         <v>0</v>
@@ -16138,7 +16141,7 @@
         <v>1644.31</v>
       </c>
       <c r="P31">
-        <v>2027.17</v>
+        <v>2100.16</v>
       </c>
       <c r="Q31">
         <v>0</v>
@@ -16215,7 +16218,7 @@
         <v>251.68</v>
       </c>
       <c r="P32">
-        <v>517.14</v>
+        <v>530.04</v>
       </c>
       <c r="Q32">
         <v>0</v>
@@ -16369,7 +16372,7 @@
         <v>508.18</v>
       </c>
       <c r="P34">
-        <v>66.7</v>
+        <v>86.4</v>
       </c>
       <c r="Q34">
         <v>0</v>
@@ -16446,7 +16449,7 @@
         <v>548.19000000000005</v>
       </c>
       <c r="P35">
-        <v>114.6</v>
+        <v>758.05</v>
       </c>
       <c r="Q35">
         <v>0</v>
@@ -17370,7 +17373,7 @@
         <v>0</v>
       </c>
       <c r="P47">
-        <v>163</v>
+        <v>959.3</v>
       </c>
       <c r="Q47">
         <v>0</v>
@@ -17447,7 +17450,7 @@
         <v>423.9</v>
       </c>
       <c r="P48">
-        <v>579.05999999999995</v>
+        <v>619.61</v>
       </c>
       <c r="Q48">
         <v>0</v>
@@ -17524,7 +17527,7 @@
         <v>6771.6</v>
       </c>
       <c r="P49">
-        <v>907.53</v>
+        <v>991.28</v>
       </c>
       <c r="Q49">
         <v>0</v>
@@ -17601,7 +17604,7 @@
         <v>1756.31</v>
       </c>
       <c r="P50">
-        <v>441.39</v>
+        <v>505.85</v>
       </c>
       <c r="Q50">
         <v>0</v>
@@ -17678,7 +17681,7 @@
         <v>392.52</v>
       </c>
       <c r="P51">
-        <v>49.3</v>
+        <v>65.3</v>
       </c>
       <c r="Q51">
         <v>0</v>
@@ -17832,7 +17835,7 @@
         <v>475.55</v>
       </c>
       <c r="P53">
-        <v>29.94</v>
+        <v>74.64</v>
       </c>
       <c r="Q53">
         <v>0</v>
@@ -17986,7 +17989,7 @@
         <v>6968.14</v>
       </c>
       <c r="P55">
-        <v>731.48</v>
+        <v>743.18</v>
       </c>
       <c r="Q55">
         <v>0</v>
@@ -18063,7 +18066,7 @@
         <v>351.6</v>
       </c>
       <c r="P56">
-        <v>936.84</v>
+        <v>1244.1199999999999</v>
       </c>
       <c r="Q56">
         <v>0</v>
@@ -18140,7 +18143,7 @@
         <v>275.2</v>
       </c>
       <c r="P57">
-        <v>281.3</v>
+        <v>334.8</v>
       </c>
       <c r="Q57">
         <v>0</v>
@@ -18294,7 +18297,7 @@
         <v>1453.89</v>
       </c>
       <c r="P59">
-        <v>492.81</v>
+        <v>667.68</v>
       </c>
       <c r="Q59">
         <v>0</v>
@@ -18371,7 +18374,7 @@
         <v>87.73</v>
       </c>
       <c r="P60">
-        <v>245.3</v>
+        <v>266.25</v>
       </c>
       <c r="Q60">
         <v>0</v>
@@ -19064,7 +19067,7 @@
         <v>1528.85</v>
       </c>
       <c r="P69">
-        <v>1238.8</v>
+        <v>2994.32</v>
       </c>
       <c r="Q69">
         <v>0</v>
@@ -19295,7 +19298,7 @@
         <v>806.7</v>
       </c>
       <c r="P72">
-        <v>579.29999999999995</v>
+        <v>699.1</v>
       </c>
       <c r="Q72">
         <v>0</v>
@@ -19372,7 +19375,7 @@
         <v>2564.08</v>
       </c>
       <c r="P73">
-        <v>331.3</v>
+        <v>946.13</v>
       </c>
       <c r="Q73">
         <v>0</v>
@@ -19449,7 +19452,7 @@
         <v>3205.26</v>
       </c>
       <c r="P74">
-        <v>850.52</v>
+        <v>1296.3599999999999</v>
       </c>
       <c r="Q74">
         <v>0</v>
@@ -19526,7 +19529,7 @@
         <v>5782.77</v>
       </c>
       <c r="P75">
-        <v>882.29</v>
+        <v>1352.67</v>
       </c>
       <c r="Q75">
         <v>0</v>
@@ -19603,7 +19606,7 @@
         <v>360.6</v>
       </c>
       <c r="P76">
-        <v>117.8</v>
+        <v>163.25</v>
       </c>
       <c r="Q76">
         <v>0</v>
@@ -19757,7 +19760,7 @@
         <v>276.93</v>
       </c>
       <c r="P78">
-        <v>150.47999999999999</v>
+        <v>209.83</v>
       </c>
       <c r="Q78">
         <v>0</v>
@@ -19911,7 +19914,7 @@
         <v>7670.07</v>
       </c>
       <c r="P80">
-        <v>2479.83</v>
+        <v>4804.8999999999996</v>
       </c>
       <c r="Q80">
         <v>0</v>
@@ -19988,7 +19991,7 @@
         <v>3574.39</v>
       </c>
       <c r="P81">
-        <v>664.76</v>
+        <v>2210.5100000000002</v>
       </c>
       <c r="Q81">
         <v>0</v>
@@ -20065,7 +20068,7 @@
         <v>799.37</v>
       </c>
       <c r="P82">
-        <v>552.47</v>
+        <v>603.72</v>
       </c>
       <c r="Q82">
         <v>0</v>
@@ -20219,7 +20222,7 @@
         <v>2160.71</v>
       </c>
       <c r="P84">
-        <v>1177.83</v>
+        <v>2207.09</v>
       </c>
       <c r="Q84">
         <v>0</v>
@@ -20296,7 +20299,7 @@
         <v>5356.76</v>
       </c>
       <c r="P85">
-        <v>2421.7399999999998</v>
+        <v>3423.97</v>
       </c>
       <c r="Q85">
         <v>0</v>
@@ -21374,7 +21377,7 @@
         <v>32.49</v>
       </c>
       <c r="P99">
-        <v>0.01</v>
+        <v>78.959999999999994</v>
       </c>
       <c r="Q99">
         <v>0</v>
@@ -21682,7 +21685,7 @@
         <v>0</v>
       </c>
       <c r="P103">
-        <v>0</v>
+        <v>5.56</v>
       </c>
       <c r="Q103">
         <v>0</v>
@@ -21913,7 +21916,7 @@
         <v>64.069999999999993</v>
       </c>
       <c r="P106">
-        <v>0</v>
+        <v>4.96</v>
       </c>
       <c r="Q106">
         <v>0</v>
@@ -23222,7 +23225,7 @@
         <v>203.03</v>
       </c>
       <c r="P123">
-        <v>17.89</v>
+        <v>21.49</v>
       </c>
       <c r="Q123">
         <v>0</v>
@@ -23299,7 +23302,7 @@
         <v>540.03</v>
       </c>
       <c r="P124">
-        <v>207.8</v>
+        <v>215.71</v>
       </c>
       <c r="Q124">
         <v>0</v>
@@ -23376,7 +23379,7 @@
         <v>788.08</v>
       </c>
       <c r="P125">
-        <v>241.87</v>
+        <v>253.37</v>
       </c>
       <c r="Q125">
         <v>0</v>
@@ -23453,7 +23456,7 @@
         <v>349.1</v>
       </c>
       <c r="P126">
-        <v>224.6</v>
+        <v>251.5</v>
       </c>
       <c r="Q126">
         <v>0</v>
@@ -23838,7 +23841,7 @@
         <v>128.09</v>
       </c>
       <c r="P131">
-        <v>466.05</v>
+        <v>572.65</v>
       </c>
       <c r="Q131">
         <v>0</v>
@@ -24069,7 +24072,7 @@
         <v>347.7</v>
       </c>
       <c r="P134">
-        <v>193.03</v>
+        <v>234.83</v>
       </c>
       <c r="Q134">
         <v>0</v>
@@ -25147,7 +25150,7 @@
         <v>449.41</v>
       </c>
       <c r="P148">
-        <v>436.87</v>
+        <v>482.17</v>
       </c>
       <c r="Q148">
         <v>0</v>
@@ -25224,7 +25227,7 @@
         <v>1131.74</v>
       </c>
       <c r="P149">
-        <v>304.58999999999997</v>
+        <v>347.79</v>
       </c>
       <c r="Q149">
         <v>0</v>
@@ -25301,7 +25304,7 @@
         <v>989.68</v>
       </c>
       <c r="P150">
-        <v>563.29999999999995</v>
+        <v>593.75</v>
       </c>
       <c r="Q150">
         <v>0</v>
@@ -25686,7 +25689,7 @@
         <v>1212.5</v>
       </c>
       <c r="P155">
-        <v>129.5</v>
+        <v>299.39999999999998</v>
       </c>
       <c r="Q155">
         <v>0</v>
@@ -25763,7 +25766,7 @@
         <v>1217.27</v>
       </c>
       <c r="P156">
-        <v>199.18</v>
+        <v>213.08</v>
       </c>
       <c r="Q156">
         <v>0</v>
@@ -25994,7 +25997,7 @@
         <v>332.2</v>
       </c>
       <c r="P159">
-        <v>470.95</v>
+        <v>482.65</v>
       </c>
       <c r="Q159">
         <v>0</v>
@@ -26071,7 +26074,7 @@
         <v>282.8</v>
       </c>
       <c r="P160">
-        <v>313.75</v>
+        <v>576.54999999999995</v>
       </c>
       <c r="Q160">
         <v>0</v>
@@ -28689,7 +28692,7 @@
         <v>10911.5</v>
       </c>
       <c r="P194">
-        <v>7867.21</v>
+        <v>24876.79</v>
       </c>
       <c r="Q194">
         <v>0</v>
@@ -28920,7 +28923,7 @@
         <v>9643.9500000000007</v>
       </c>
       <c r="P197">
-        <v>4716.7</v>
+        <v>5779.94</v>
       </c>
       <c r="Q197">
         <v>0</v>
@@ -28997,7 +29000,7 @@
         <v>7099.57</v>
       </c>
       <c r="P198">
-        <v>5330.29</v>
+        <v>9705.77</v>
       </c>
       <c r="Q198">
         <v>0</v>
@@ -29074,7 +29077,7 @@
         <v>10437.030000000001</v>
       </c>
       <c r="P199">
-        <v>8063.34</v>
+        <v>9755.67</v>
       </c>
       <c r="Q199">
         <v>0</v>
@@ -29151,7 +29154,7 @@
         <v>14032.28</v>
       </c>
       <c r="P200">
-        <v>10665.79</v>
+        <v>15322.7</v>
       </c>
       <c r="Q200">
         <v>0</v>
@@ -29228,7 +29231,7 @@
         <v>819.93</v>
       </c>
       <c r="P201">
-        <v>649.42999999999995</v>
+        <v>1161.1600000000001</v>
       </c>
       <c r="Q201">
         <v>0</v>
@@ -29382,7 +29385,7 @@
         <v>1498.34</v>
       </c>
       <c r="P203">
-        <v>1403.55</v>
+        <v>5223.99</v>
       </c>
       <c r="Q203">
         <v>0</v>
@@ -29459,7 +29462,7 @@
         <v>2807.35</v>
       </c>
       <c r="P204">
-        <v>1867.65</v>
+        <v>3277.5</v>
       </c>
       <c r="Q204">
         <v>0</v>
@@ -29536,7 +29539,7 @@
         <v>153570.17000000001</v>
       </c>
       <c r="P205">
-        <v>80514.02</v>
+        <v>109524.39</v>
       </c>
       <c r="Q205">
         <v>0</v>
@@ -29613,7 +29616,7 @@
         <v>11988.76</v>
       </c>
       <c r="P206">
-        <v>6680.78</v>
+        <v>9043.35</v>
       </c>
       <c r="Q206">
         <v>0</v>
@@ -29690,7 +29693,7 @@
         <v>3782.99</v>
       </c>
       <c r="P207">
-        <v>728.05</v>
+        <v>783.75</v>
       </c>
       <c r="Q207">
         <v>0</v>
@@ -29767,7 +29770,7 @@
         <v>2317.5500000000002</v>
       </c>
       <c r="P208">
-        <v>290</v>
+        <v>433</v>
       </c>
       <c r="Q208">
         <v>0</v>
@@ -29844,7 +29847,7 @@
         <v>8450.7999999999993</v>
       </c>
       <c r="P209">
-        <v>3988.82</v>
+        <v>5353.31</v>
       </c>
       <c r="Q209">
         <v>0</v>
@@ -29921,7 +29924,7 @@
         <v>20216.419999999998</v>
       </c>
       <c r="P210">
-        <v>16613.75</v>
+        <v>29217.46</v>
       </c>
       <c r="Q210">
         <v>0</v>
@@ -30614,7 +30617,7 @@
         <v>5408.2</v>
       </c>
       <c r="P219">
-        <v>1786.26</v>
+        <v>6246.19</v>
       </c>
       <c r="Q219">
         <v>0</v>
@@ -30845,7 +30848,7 @@
         <v>2431.15</v>
       </c>
       <c r="P222">
-        <v>5449.8</v>
+        <v>6642.2</v>
       </c>
       <c r="Q222">
         <v>0</v>
@@ -30922,7 +30925,7 @@
         <v>2748.05</v>
       </c>
       <c r="P223">
-        <v>3777.22</v>
+        <v>4725.95</v>
       </c>
       <c r="Q223">
         <v>0</v>
@@ -30999,7 +31002,7 @@
         <v>5884.89</v>
       </c>
       <c r="P224">
-        <v>2263.23</v>
+        <v>3883.83</v>
       </c>
       <c r="Q224">
         <v>0</v>
@@ -31076,7 +31079,7 @@
         <v>5304.37</v>
       </c>
       <c r="P225">
-        <v>9542.5</v>
+        <v>12189.58</v>
       </c>
       <c r="Q225">
         <v>0</v>
@@ -31153,7 +31156,7 @@
         <v>630.75</v>
       </c>
       <c r="P226">
-        <v>306.55</v>
+        <v>401.36</v>
       </c>
       <c r="Q226">
         <v>0</v>
@@ -31307,7 +31310,7 @@
         <v>2586.27</v>
       </c>
       <c r="P228">
-        <v>2485.46</v>
+        <v>3183.25</v>
       </c>
       <c r="Q228">
         <v>0</v>
@@ -31384,7 +31387,7 @@
         <v>3384.9</v>
       </c>
       <c r="P229">
-        <v>581.79999999999995</v>
+        <v>933.45</v>
       </c>
       <c r="Q229">
         <v>0</v>
@@ -31461,7 +31464,7 @@
         <v>18556.27</v>
       </c>
       <c r="P230">
-        <v>21101.45</v>
+        <v>32367.51</v>
       </c>
       <c r="Q230">
         <v>0</v>
@@ -31538,7 +31541,7 @@
         <v>4790.9799999999996</v>
       </c>
       <c r="P231">
-        <v>4777.58</v>
+        <v>5632.88</v>
       </c>
       <c r="Q231">
         <v>0</v>
@@ -31615,7 +31618,7 @@
         <v>2022.35</v>
       </c>
       <c r="P232">
-        <v>1928.74</v>
+        <v>2400.84</v>
       </c>
       <c r="Q232">
         <v>0</v>
@@ -31769,7 +31772,7 @@
         <v>2024.05</v>
       </c>
       <c r="P234">
-        <v>2746.48</v>
+        <v>3953.57</v>
       </c>
       <c r="Q234">
         <v>0</v>
@@ -31846,7 +31849,7 @@
         <v>10644.94</v>
       </c>
       <c r="P235">
-        <v>7410.16</v>
+        <v>9696.7800000000007</v>
       </c>
       <c r="Q235">
         <v>0</v>
@@ -32539,7 +32542,7 @@
         <v>3516.16</v>
       </c>
       <c r="P244">
-        <v>2730.14</v>
+        <v>4491.96</v>
       </c>
       <c r="Q244">
         <v>0</v>
@@ -32770,7 +32773,7 @@
         <v>1706.35</v>
       </c>
       <c r="P247">
-        <v>3425.04</v>
+        <v>4092.26</v>
       </c>
       <c r="Q247">
         <v>0</v>
@@ -32847,7 +32850,7 @@
         <v>4351.96</v>
       </c>
       <c r="P248">
-        <v>2342.2600000000002</v>
+        <v>3180.69</v>
       </c>
       <c r="Q248">
         <v>0</v>
@@ -32924,7 +32927,7 @@
         <v>6772.9</v>
       </c>
       <c r="P249">
-        <v>9462.0300000000007</v>
+        <v>10828.19</v>
       </c>
       <c r="Q249">
         <v>0</v>
@@ -33001,7 +33004,7 @@
         <v>10251.93</v>
       </c>
       <c r="P250">
-        <v>8491.7800000000007</v>
+        <v>10434.879999999999</v>
       </c>
       <c r="Q250">
         <v>0</v>
@@ -33078,7 +33081,7 @@
         <v>1478.26</v>
       </c>
       <c r="P251">
-        <v>557.72</v>
+        <v>716.95</v>
       </c>
       <c r="Q251">
         <v>0</v>
@@ -33232,7 +33235,7 @@
         <v>3188.47</v>
       </c>
       <c r="P253">
-        <v>740.1</v>
+        <v>1438.9</v>
       </c>
       <c r="Q253">
         <v>0</v>
@@ -33386,7 +33389,7 @@
         <v>29857.48</v>
       </c>
       <c r="P255">
-        <v>19624.55</v>
+        <v>26068.95</v>
       </c>
       <c r="Q255">
         <v>0</v>
@@ -33463,7 +33466,7 @@
         <v>6679.21</v>
       </c>
       <c r="P256">
-        <v>5071.66</v>
+        <v>5420.08</v>
       </c>
       <c r="Q256">
         <v>0</v>
@@ -33540,7 +33543,7 @@
         <v>3019.73</v>
       </c>
       <c r="P257">
-        <v>1557.26</v>
+        <v>1691.66</v>
       </c>
       <c r="Q257">
         <v>0</v>
@@ -33694,7 +33697,7 @@
         <v>4746.4399999999996</v>
       </c>
       <c r="P259">
-        <v>2570.84</v>
+        <v>4220.72</v>
       </c>
       <c r="Q259">
         <v>0</v>
@@ -33771,7 +33774,7 @@
         <v>18146.46</v>
       </c>
       <c r="P260">
-        <v>13052.18</v>
+        <v>22736.11</v>
       </c>
       <c r="Q260">
         <v>0</v>
@@ -35957,7 +35960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A289" t="str">
         <v xml:space="preserve">VENDEDOR </v>
       </c>
@@ -36034,7 +36037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A290" t="str">
         <v xml:space="preserve">VENDEDOR </v>
       </c>
@@ -36111,7 +36114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A291" t="str">
         <v xml:space="preserve">VENDEDOR </v>
       </c>
@@ -36188,7 +36191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>0</v>
       </c>
@@ -36262,6 +36265,163 @@
         <v>0</v>
       </c>
       <c r="Y292">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="299" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="B299" t="s">
+        <v>13</v>
+      </c>
+      <c r="C299">
+        <f t="shared" ref="C299:AN299" si="0">SUM(C17:C292)</f>
+        <v>642279.78</v>
+      </c>
+      <c r="D299">
+        <f t="shared" si="0"/>
+        <v>619860.11</v>
+      </c>
+      <c r="E299">
+        <f t="shared" si="0"/>
+        <v>618508.72</v>
+      </c>
+      <c r="F299">
+        <f t="shared" si="0"/>
+        <v>667531.78999999992</v>
+      </c>
+      <c r="G299">
+        <f t="shared" si="0"/>
+        <v>686623.00000000023</v>
+      </c>
+      <c r="H299">
+        <f t="shared" si="0"/>
+        <v>536152.02000000025</v>
+      </c>
+      <c r="I299">
+        <f t="shared" si="0"/>
+        <v>691743.53</v>
+      </c>
+      <c r="J299">
+        <f t="shared" si="0"/>
+        <v>573251.49</v>
+      </c>
+      <c r="K299">
+        <f t="shared" si="0"/>
+        <v>648519.03000000014</v>
+      </c>
+      <c r="L299">
+        <f t="shared" si="0"/>
+        <v>663917.68999999971</v>
+      </c>
+      <c r="M299">
+        <f t="shared" si="0"/>
+        <v>594261.41</v>
+      </c>
+      <c r="N299">
+        <f t="shared" si="0"/>
+        <v>545469.44999999995</v>
+      </c>
+      <c r="O299">
+        <f t="shared" si="0"/>
+        <v>505083.35</v>
+      </c>
+      <c r="P299">
+        <f t="shared" si="0"/>
+        <v>472249.95000000019</v>
+      </c>
+      <c r="Q299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Y299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AB299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AD299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AF299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AG299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AH299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AI299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AJ299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AK299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AL299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AM299">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AN299">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>